<commit_message>
Export: split outbound sheet into Initial / Follow-up 8.26 tabs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/Diligence Question Responses/Diligence Responses_20260909.xlsx
+++ b/Diligence Question Responses/Diligence Responses_20260909.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Diligence Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Initial Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Follow-up Questions 8.26" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -439,7 +440,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Diligence Questions</t>
+          <t>Diligence Questions — initial list (responses sent 2026-08-05)</t>
         </is>
       </c>
     </row>
@@ -928,33 +929,94 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Follow-up Questions — fund email 2026-08-26 (items 6-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Diligence question / request</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Response / evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Installment purchase — economics walkthrough</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>1. Could you walk us through the economics of a typical installment purchase, from the swipe through to final payment? We're mainly after the revenue lines and their timing: what you earn on the transaction itself (interchange, net of network and processor costs), what's charged upfront at origination, and what accrues over the term.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>At the swipe, Zed earns interchange on these purchases like any other purchase (net interchange economics covered in 11). In fact, because purchases are enrolled in installments post purchase, there is no way to distinguish purchases that will ultimately be enrolled in installments and those that won't at the time of the swipe. Our installment feature works much like AmEx's "Pay Over Time": after a purchase, certain transactions are eligible for installment enrollment and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
 Upon enrollment: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
@@ -963,65 +1025,65 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Installment purchase — flow of funds</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1 (cont.): Plus the flow of funds: who pays whom, when, and which entity each flow lands in.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>See the Installment Funds Flow diagram in Data Room / Product.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Revolver and pay-in-full — economics walkthrough</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>2. Do the same walkthrough for a revolving balance and for a pay-in-full statement, so we can see how the three products differ economically.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Just to clarify: today, "pay in full" and "revolving" are two payment behaviors on the same card rather than separate products. Paying in full was the required dynamic of our original charge card, which we have since retired. We launched revolving on May 25th; the first statements carrying a Minimum Payment Due below the statement ending balance were generated June 1, and the second and final cohort of users still on the charge-card dynamic (where the MPD equaled the statement ending balance) transitioned on June 15. Since then, our entire customer base is on the revolving product. Cardholders can of course still choose to pay their balance in full each cycle to avoid interest — like any credit card — but it's no longer required. So the walkthrough below covers our sole card product, a revolving credit card with an installment feature.
 Interchange: as in 6.1, every purchase earns Zed interchange at the swipe — payment behavior plays out afterwards and never changes the transaction-level economics.
@@ -1040,355 +1102,355 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>"Installment fees" field definition</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>3. Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Installment fees in the tape include upfront fees and the "termination fee". Just to reiterate, to the user, "termination fees" are actually just an accelerated billing of the final (i.e. cancellation cycle's) interest. They don't see it as a "termination fee", but rather final period interest. Unfortunately, per our ledger/system of record, we have to classify these as fees rather than interest. You should find even more detail about the installment charges in the installment tape that we provided, where we break out every installment plan and associated fees.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Fee schedule — rates and formula</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>4. Confirm the fee schedule: add-on rate by tenor, and the origination fee formula. We have been told 0.5% × number of months (3% on a 6-month term). Confirm or correct.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Confirmed. The upfront fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms). The add-on rate is 1% of original principal per month, so by the end of the term, customers will pay 3% for a 3-month, 6% for 6-month, 12% for 12-month terms. The difference is that the upfront fee is billed entirely in the enrollment/first cycle and the add-on rate is billed each cycle of the term at the 1% times original principal amount.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Fee schedule — netted vs financed</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>4 (cont.): Is the fee netted from the disbursement or financed into the balance?</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the upfront fee is charged to the account and billed on the first statement.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>9.3</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Fee schedule — prepayment refund and interest rebate</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>4 (cont.): Is it refundable on prepayment, and is unearned add-on interest rebated?</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>If a plan is terminated in the first month, the upfront fee is reversed and no termination fee applies; after the first month, the upfront fee is retained and a termination fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).
 Prepayment cannot be done automatically. A user must explicitly end/cancel a plan, all billing of the remaining principal will be accelerated and the termination fee (final period interest) will be applied if it's any cycle other than the enrollment cycle.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Revenue fields absent from the tape</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>5. The tape shows late fees and installment fees but no interchange, no annual fee, no upfront fee, no cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. Zed does not charge annual fees nor do we allow cash advances. Late fees, installment enrollment upfront fees and installment termination fees (i.e. final period interest) are the only fees that Zed charges.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Net interchange as % of GMV</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>6. What is your net interchange as a percentage of GMV for the last six months (if possible, split domestic vs international)?</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Blended Average: 1.43%; Domestic: 1.17%; International: 1.84%</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>BSP ceilings — headroom confirmation</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>7. Both your revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom.</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. That being said, Zed, other issuers and the Credit Card Association of the Philippines (CCAP) are all actively involved in discussions with the BSP around the re-evaluation of the current caps.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>12.2</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>BSP ceilings — cut sensitivity</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>7 (cont.): …and tell us what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Preface: it is incredibly unlikely that the BSP will reduce the cap on credit card interest rates further. The BSP has received significant pressure from Banks to raise this cap, which was originally imposed in 2020 as a result of COVID. As a matter of pattern and direction, the BSP most recently increased the cap in 2023 from 2% to the current level of 3% per month.
 Re: the impact of a rate reduction, we previously shared a breakdown of unit economics in response to item 2.3. The Pro Forma column in this file indicates the steady state revenue earned from interest on a per user basis. Even if this revolving interest revenue drops down to zero (i.e. a 0% interest rate), our users are still marginally profitable on the basis of interchange and installment conversions alone. This, of course, assumes no debt expense. So the logical floor of interest rate cap that we could support is almost directly equivalent to our borrowing costs because we're close to breakeven without any interest revenue and no debt financing assumed.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>13.1</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Loss figure — basis and denominator</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>8. What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator?</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume. We manage to a 1–3% target range and are currently at 1.82%, in line with US prime credit card benchmarks.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>13.2</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Charge-off policy and changes since launch</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>8 (cont.): We'd also appreciate your charge-off policy in DPD, and any change to it since launch.</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Drafted</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Restructures and re-aging</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>8 (cont.): …and your approach to restructures/re-aging.</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Re-aging to Current requires all arrears cleared. No restructuring plan currently exists. Certain accounts that are &gt;15 DPD are eligible to enroll into a payment plan. Once this plan is completed, though, the accounts are wound down and they cannot continue to be Zed customers.</t>
         </is>

</xml_diff>

<commit_message>
Export styling matches the 8/5 sheet: navy banner, blue headers, section grouping
Follow-up tab groups by email bullet (Section = 'Email question N', N mapped
back to Raymond's 1-8); status fills peach for Closed, gray flags non-Closed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/Diligence Question Responses/Diligence Responses_20260909.xlsx
+++ b/Diligence Question Responses/Diligence Responses_20260909.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,22 +27,90 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="18"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF17365D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF17365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B9BD5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -50,16 +118,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="medium"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,115 +541,115 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Diligence Questions — initial list (responses sent 2026-08-05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+          <t>Diligence Questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Diligence question / request</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Response / evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Revolving credit — launch and economics</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Launch date</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Launch date for revolving credit?</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>May 25th; first statement end dates with minimum balances due were June 1 and June 15.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Revolving credit — launch and economics</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Launch date</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Launch date for revolving credit?</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>May 25th; first statement end dates with minimum balances due were June 1 and June 15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Revolving credit — launch and economics</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>APR, minimum payment and eligibility</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Target APR, minimum payment formula, and eligibility criteria at launch. Does the full book qualify on day one, or selected cohorts/score bands only?</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>APR for all customers is 3% monthly.
 All accounts were eligible at launch, but past-due balances were still considered past-due. Only charges after revolving launched were able to revolve.
@@ -542,97 +657,97 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Revolving credit — launch and economics</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Adoption / balance mix</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Expected share of balances revolving at month 6 and month 12 post-launch?</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>~23% of the base is revolving as of July. We expect the share of revolvers will rise over the next year and we are tracking it closely</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Revolving credit — launch and economics</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Provisioning and delinquency treatment</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Provisioning approach for revolving balances, and how the credit policy treats a revolver that subsequently goes delinquent (limit freeze, re-age rules, minimum-payment escalation).</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Zed applies a single Net Flow Rate provisioning methodology across all balances with segmentation driven by days past due rather than product type (there is only one product type), so revolving balances flow through the same eight DPD buckets (Current through 181+) as installment loans. Once a revolver becomes past due, we apply a hard card freeze at DPD 1. Zed reserves the right to collect the entire balance in such an event. Re-aging to Current requires all arrears cleared.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Asset economics — pre- and post-revolving</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Installment fee economics and cancellations</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Installments are 18.2% of the June 30 book at a ~7.2% blended fee on volume, with ~11% of originated volume cancelled. Term distribution behind the blended fee, and fee treatment on cancellation (refunded or retained)?</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>See attached for a revised statement tape including installment conversions. The blended installment charges are ~3.2%, and cancellations are ~5.1% of originated volume. Cancellations contain past due-related accelerations (6 DPD) and customer initiated "end plan early" availments. The ~3.2% installment charges includes upfront fees and current month interest (cancellation fee).
 If an installment is 'cancelled' in the first month, the initial upfront fee is reversed and there is no cancellation fee. Otherwise, the cancellation fee is equal to that month's interest, and the upfront fee remains.
@@ -640,296 +755,299 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Asset economics — pre- and post-revolving</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Plan mechanics and performance</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>The June 30 tape shows every account with a live installment balance as Current — we assume plans are cancelled or accelerated into the statement balance on delinquency. Confirm the mechanics, and provide delinquency and loss performance on a plan-level basis.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Correct on the mechanics - additional detail on installment loans to be provided.
 Installment loans and associated terms do not exist indepedently of the credit card balance. Installments are billed on the credit card statement cycles. Once billed, they are technically added to the purchase/revolving balance. Because of our min payment rules, we expect full payment of the installment billing by the due date in order to keep the account in good standing. But it is technically not possible to delinquent on an installment plan independent of the credit card, because they're all part of the same expected minimum payment and credit card product.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Asset economics — pre- and post-revolving</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Unit economics</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Unit economics per active account today (interchange, installment fees, late fees, less credit cost and processing cost), and the same view pro forma with revolving at your base-case adoption.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>See attached for current and PF unit economics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Underwriting and credit risk</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Cohort delinquency drivers and target losses</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>2024Q3–2025Q2 cohorts show 10–25% of accounts ever reaching 90+ DPD — high for a prime positioning. What drove this, what changed, and what is the target loss rate for 2026 vintages at the re-leveled limits?</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Earlier cohorts (Q3 2024's N=100) are too small to infer anything meaningful (these were our very first issuances beyond friends and family). Q2 2025 (N=1,087) is a larger cohort with 9.8% currently 90+ DPD but still small as we begin adding thousands of cardholders per quarter going forward. Improvements in past due rates are a result of model refinements in Q3 and Q4 2025 as we began incorporating actual performance to better inform probability of default.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Underwriting and credit risk</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Cohort delinquency drivers and target losses</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>2024Q3–2025Q2 cohorts show 10–25% of accounts ever reaching 90+ DPD — high for a prime positioning. What drove this, what changed, and what is the target loss rate for 2026 vintages at the re-leveled limits?</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Earlier cohorts (Q3 2024's N=100) are too small to infer anything meaningful (these were our very first issuances beyond friends and family). Q2 2025 (N=1,087) is a larger cohort with 9.8% currently 90+ DPD but still small as we begin adding thousands of cardholders per quarter going forward. Improvements in past due rates are a result of model refinements in Q3 and Q4 2025 as we began incorporating actual performance to better inform probability of default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Underwriting and credit risk</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Limit re-leveling guardrails</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Credit limit re-leveling raised the median limit from PHP 35K to PHP 50K in March 2026. What guardrails cap exposure growth for accounts with limited payment history, and how will limits interact with revolving eligibility?</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>We don't increase credit limits for accounts that have ever had a serious past due balances (15+ DPD per our current policy). We set small initial limits that increase as cardholders display positive payment history. The initial line is set at min(ADB, 2x income) today; it was 1x income until March 23, 2026. We did a portfolio wide reevaluation of CLs in preparation for installment and revolving launch and are comfortable with our current policy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Charge-off, collections, and recoveries</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Charge-off policy</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>The June 30 tape carries PHP 11.1M of 180+ DPD with no write-off. What is the charge-off policy (we would expect write-off at 180 DPD), and when will a written policy be adopted?</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>In line with our ECL policy, we have set-up 100% provisioning for accounts that are 180+ DPD. We have not officially written anything off due to resource constraints. As an early-stage company with a lean PH team, we have not yet stood up the collections-substantiation and BIR documentation process required to write off (the tax code worthlessness tests require documented, exhausted collection efforts per account). We are building this process out.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Charge-off, collections, and recoveries</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Charge-off policy</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>The June 30 tape carries PHP 11.1M of 180+ DPD with no write-off. What is the charge-off policy (we would expect write-off at 180 DPD), and when will a written policy be adopted?</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>In line with our ECL policy, we have set-up 100% provisioning for accounts that are 180+ DPD. We have not officially written anything off due to resource constraints. As an early-stage company with a lean PH team, we have not yet stood up the collections-substantiation and BIR documentation process required to write off (the tax code worthlessness tests require documented, exhausted collection efforts per account). We are building this process out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Charge-off, collections, and recoveries</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Recoveries</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Recoveries achieved on 90+ DPD balances to date?</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Provided — see the "90+ Recovery Summary" tab added to the statement tape, with trace-back columns on the original tape so the derivation is auditable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Data requested</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Payment-level tape</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>To discuss.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Data requested</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Payment-level tape</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>To discuss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Data requested</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Installment plan tape</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Per installment plan: plan ID, origination date, term, fee, status, cancellation/acceleration date and reason.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Provided — plan-level installment tape (plan ID, opt-in date, tenure, upfront fee, monthly interest, status by month, termination date/source), also in Data Room / Loan Tape.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Data requested</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Cohort performance file</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Per cohort: monthly origination, outstanding, and cumulative gross/net loss by MOB, split purchase vs. installment.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>The loan tape shows unique cardholders and their origination cohort, which can be joined with the statement tape to show, by unique cardholder, statement charges and credits. We added gross installment conversions as well. DPD columns show what statements balances ever went past due or are currently past due. The statement data can be used to reconstruct every unique cardholders charges and payment history by using the UID key.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -940,83 +1058,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Follow-up Questions — fund email 2026-08-26 (items 6-13)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+          <t>Follow-up Questions (email 8/26/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Diligence question / request</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Response / evidence</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Email question 1</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Installment purchase — economics walkthrough</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>1. Could you walk us through the economics of a typical installment purchase, from the swipe through to final payment? We're mainly after the revenue lines and their timing: what you earn on the transaction itself (interchange, net of network and processor costs), what's charged upfront at origination, and what accrues over the term.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>At the swipe, Zed earns interchange on these purchases like any other purchase (net interchange economics covered in 11). In fact, because purchases are enrolled in installments post purchase, there is no way to distinguish purchases that will ultimately be enrolled in installments and those that won't at the time of the swipe. Our installment feature works much like AmEx's "Pay Over Time": after a purchase, certain transactions are eligible for installment enrollment and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
 Upon enrollment: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
@@ -1025,65 +1143,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Email question 1</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Installment purchase — flow of funds</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>1 (cont.): Plus the flow of funds: who pays whom, when, and which entity each flow lands in.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>See the Installment Funds Flow diagram in Data Room / Product.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Email question 2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Revolver and pay-in-full — economics walkthrough</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>2. Do the same walkthrough for a revolving balance and for a pay-in-full statement, so we can see how the three products differ economically.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Just to clarify: today, "pay in full" and "revolving" are two payment behaviors on the same card rather than separate products. Paying in full was the required dynamic of our original charge card, which we have since retired. We launched revolving on May 25th; the first statements carrying a Minimum Payment Due below the statement ending balance were generated June 1, and the second and final cohort of users still on the charge-card dynamic (where the MPD equaled the statement ending balance) transitioned on June 15. Since then, our entire customer base is on the revolving product. Cardholders can of course still choose to pay their balance in full each cycle to avoid interest — like any credit card — but it's no longer required. So the walkthrough below covers our sole card product, a revolving credit card with an installment feature.
 Interchange: as in 6.1, every purchase earns Zed interchange at the swipe — payment behavior plays out afterwards and never changes the transaction-level economics.
@@ -1102,361 +1220,364 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>"Installment fees" field definition</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>3. Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Installment fees in the tape include upfront fees and the "termination fee". Just to reiterate, to the user, "termination fees" are actually just an accelerated billing of the final (i.e. cancellation cycle's) interest. They don't see it as a "termination fee", but rather final period interest. Unfortunately, per our ledger/system of record, we have to classify these as fees rather than interest. You should find even more detail about the installment charges in the installment tape that we provided, where we break out every installment plan and associated fees.</t>
-        </is>
-      </c>
-    </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Fee schedule — rates and formula</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>4. Confirm the fee schedule: add-on rate by tenor, and the origination fee formula. We have been told 0.5% × number of months (3% on a 6-month term). Confirm or correct.</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed. The upfront fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms). The add-on rate is 1% of original principal per month, so by the end of the term, customers will pay 3% for a 3-month, 6% for 6-month, 12% for 12-month terms. The difference is that the upfront fee is billed entirely in the enrollment/first cycle and the add-on rate is billed each cycle of the term at the 1% times original principal amount.</t>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Email question 3</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>"Installment fees" field definition</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>3. Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Installment fees in the tape include upfront fees and the "termination fee". Just to reiterate, to the user, "termination fees" are actually just an accelerated billing of the final (i.e. cancellation cycle's) interest. They don't see it as a "termination fee", but rather final period interest. Unfortunately, per our ledger/system of record, we have to classify these as fees rather than interest. You should find even more detail about the installment charges in the installment tape that we provided, where we break out every installment plan and associated fees.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Email question 4</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Fee schedule — rates and formula</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>4. Confirm the fee schedule: add-on rate by tenor, and the origination fee formula. We have been told 0.5% × number of months (3% on a 6-month term). Confirm or correct.</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed. The upfront fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms). The add-on rate is 1% of original principal per month, so by the end of the term, customers will pay 3% for a 3-month, 6% for 6-month, 12% for 12-month terms. The difference is that the upfront fee is billed entirely in the enrollment/first cycle and the add-on rate is billed each cycle of the term at the 1% times original principal amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Email question 4</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Fee schedule — netted vs financed</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>4 (cont.): Is the fee netted from the disbursement or financed into the balance?</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the upfront fee is charged to the account and billed on the first statement.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>9.3</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Email question 4</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Fee schedule — prepayment refund and interest rebate</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>4 (cont.): Is it refundable on prepayment, and is unearned add-on interest rebated?</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>If a plan is terminated in the first month, the upfront fee is reversed and no termination fee applies; after the first month, the upfront fee is retained and a termination fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).
 Prepayment cannot be done automatically. A user must explicitly end/cancel a plan, all billing of the remaining principal will be accelerated and the termination fee (final period interest) will be applied if it's any cycle other than the enrollment cycle.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Revenue fields absent from the tape</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>5. The tape shows late fees and installment fees but no interchange, no annual fee, no upfront fee, no cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. Zed does not charge annual fees nor do we allow cash advances. Late fees, installment enrollment upfront fees and installment termination fees (i.e. final period interest) are the only fees that Zed charges.</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Net interchange as % of GMV</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>6. What is your net interchange as a percentage of GMV for the last six months (if possible, split domestic vs international)?</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Blended Average: 1.43%; Domestic: 1.17%; International: 1.84%</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Email question 5</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Revenue fields absent from the tape</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>5. The tape shows late fees and installment fees but no interchange, no annual fee, no upfront fee, no cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. Zed does not charge annual fees nor do we allow cash advances. Late fees, installment enrollment upfront fees and installment termination fees (i.e. final period interest) are the only fees that Zed charges.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>BSP ceilings — headroom confirmation</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>7. Both your revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom.</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. That being said, Zed, other issuers and the Credit Card Association of the Philippines (CCAP) are all actively involved in discussions with the BSP around the re-evaluation of the current caps.</t>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Email question 6</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Net interchange as % of GMV</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>6. What is your net interchange as a percentage of GMV for the last six months (if possible, split domestic vs international)?</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Blended Average: 1.43%; Domestic: 1.17%; International: 1.84%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Email question 7</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>BSP ceilings — headroom confirmation</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>7. Both your revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom.</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. That being said, Zed, other issuers and the Credit Card Association of the Philippines (CCAP) are all actively involved in discussions with the BSP around the re-evaluation of the current caps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>12.2</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Email question 7</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>BSP ceilings — cut sensitivity</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>7 (cont.): …and tell us what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Preface: it is incredibly unlikely that the BSP will reduce the cap on credit card interest rates further. The BSP has received significant pressure from Banks to raise this cap, which was originally imposed in 2020 as a result of COVID. As a matter of pattern and direction, the BSP most recently increased the cap in 2023 from 2% to the current level of 3% per month.
 Re: the impact of a rate reduction, we previously shared a breakdown of unit economics in response to item 2.3. The Pro Forma column in this file indicates the steady state revenue earned from interest on a per user basis. Even if this revolving interest revenue drops down to zero (i.e. a 0% interest rate), our users are still marginally profitable on the basis of interchange and installment conversions alone. This, of course, assumes no debt expense. So the logical floor of interest rate cap that we could support is almost directly equivalent to our borrowing costs because we're close to breakeven without any interest revenue and no debt financing assumed.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>13.1</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Loss figure — basis and denominator</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>8. What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator?</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume. We manage to a 1–3% target range and are currently at 1.82%, in line with US prime credit card benchmarks.</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Email question 8</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Loss figure — basis and denominator</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>8. What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator?</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume. We manage to a 1–3% target range and are currently at 1.82%, in line with US prime credit card benchmarks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>13.2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Email question 8</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Charge-off policy and changes since launch</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>8 (cont.): We'd also appreciate your charge-off policy in DPD, and any change to it since launch.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>Drafted</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Follow-up questions (fund email 2026-08-26 — bullets 1–8 → items 6–13; multi-part bullets split as .1/.2/.3)</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Email question 8</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Restructures and re-aging</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>8 (cont.): …and your approach to restructures/re-aging.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Re-aging to Current requires all arrears cleared. No restructuring plan currently exists. Certain accounts that are &gt;15 DPD are eligible to enroll into a payment plan. Once this plan is completed, though, the accounts are wound down and they cannot continue to be Zed customers.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>